<commit_message>
Laminas regeneradas (regeneracion completa del 2026-10-04), piramides 2018-2024, empates nombrados (#191) (graficos_regionales_indicadores)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_indicadores/plot_regional_grupos_e_rezjov_a_2021_antofagasta_sexo.xlsx
+++ b/output/graficos_regionales_indicadores/plot_regional_grupos_e_rezjov_a_2021_antofagasta_sexo.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-10-01 15:05</t>
+    <t xml:space="preserve">2026-10-05 06:27</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -469,7 +469,7 @@
         <v>3.3</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="3">

</xml_diff>